<commit_message>
Performed anovas for CH4, N2O, GWP, and yield.
</commit_message>
<xml_diff>
--- a/Data/seasonal_total_N2O.xlsx
+++ b/Data/seasonal_total_N2O.xlsx
@@ -357,12 +357,12 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>plot_number</t>
+          <t>Plot</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>total_N2O_emissions</t>
+          <t>total_N20_emissions</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -377,7 +377,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>total_N2O_emissions_kg_ha</t>
+          <t>total_N20_emissions_kg_ha</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -413,7 +413,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>127.2033062714449</v>
+        <v>216.3353685282463</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -426,7 +426,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0.1272033062714449</v>
+        <v>0.2163353685282463</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>185.0901377227941</v>
+        <v>367.4503173691147</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0.1850901377227941</v>
+        <v>0.3674503173691147</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>287.7253768477936</v>
+        <v>641.921733997722</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>0.2877253768477936</v>
+        <v>0.641921733997722</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>115.5985868481932</v>
+        <v>671.855123315381</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>0.1155985868481932</v>
+        <v>0.671855123315381</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>72.73477338906569</v>
+        <v>2085.108347936402</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>0.0727347733890657</v>
+        <v>2.085108347936401</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>128.0882641987646</v>
+        <v>1613.258757998555</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>0.1280882641987647</v>
+        <v>1.613258757998554</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>839.1936458550648</v>
+        <v>2356.997371975801</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="E8">
-        <v>0.8391936458550648</v>
+        <v>2.356997371975802</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>265.3412323324026</v>
+        <v>1092.072979452755</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>0.2653412323324026</v>
+        <v>1.092072979452755</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>645.8277070167658</v>
+        <v>2184.234392759074</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -810,7 +810,7 @@
         </is>
       </c>
       <c r="E10">
-        <v>0.6458277070167657</v>
+        <v>2.184234392759074</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>575.9849393087039</v>
+        <v>9553.223882650849</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>0.575984939308704</v>
+        <v>9.553223882650849</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>164.7225349177046</v>
+        <v>2808.672600434861</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>0.1647225349177046</v>
+        <v>2.808672600434861</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>158.4514312819812</v>
+        <v>1720.058602968172</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="E13">
-        <v>0.1584514312819812</v>
+        <v>1.720058602968172</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>551.5277378158329</v>
+        <v>2005.072788543479</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="E14">
-        <v>0.5515277378158329</v>
+        <v>2.005072788543479</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>483.8950735352444</v>
+        <v>1485.996072705291</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="E15">
-        <v>0.4838950735352444</v>
+        <v>1.485996072705291</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>330.841463056127</v>
+        <v>983.9281216641028</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
         </is>
       </c>
       <c r="E16">
-        <v>0.330841463056127</v>
+        <v>0.9839281216641028</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
made them figure 2 and 3.
</commit_message>
<xml_diff>
--- a/Data/seasonal_total_N2O.xlsx
+++ b/Data/seasonal_total_N2O.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>671.855123315381</v>
+        <v>1099.399292697896</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>0.671855123315381</v>
+        <v>1.099399292697896</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>2085.108347936402</v>
+        <v>3157.909943599355</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>2.085108347936401</v>
+        <v>3.157909943599355</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>1613.258757998555</v>
+        <v>2491.29506831405</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>1.613258757998554</v>
+        <v>2.49129506831405</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>9553.223882650849</v>
+        <v>13401.42273430119</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>9.553223882650849</v>
+        <v>13.40142273430119</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>2808.672600434861</v>
+        <v>4252.398907986254</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>2.808672600434861</v>
+        <v>4.252398907986254</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>1720.058602968172</v>
+        <v>2461.836755428674</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="E13">
-        <v>1.720058602968172</v>
+        <v>2.461836755428674</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>

</xml_diff>